<commit_message>
Restaurando código completo con el nuevo motor de Excel
</commit_message>
<xml_diff>
--- a/plantilla_presupuesto.xlsx
+++ b/plantilla_presupuesto.xlsx
@@ -275,7 +275,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -290,6 +290,21 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
@@ -374,21 +389,6 @@
         <color indexed="64"/>
       </top>
       <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -432,11 +432,63 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -448,13 +500,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -462,31 +513,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -973,88 +1033,109 @@
       <c r="F15" s="8"/>
     </row>
     <row r="16" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="17" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="9" t="s">
+    <row r="17" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A17" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="23" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:6" s="16" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="15"/>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-    </row>
-    <row r="19" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:6" s="16" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="22" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="F22" s="17" t="s">
+    <row r="18" spans="1:6" s="24" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="26"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
+    </row>
+    <row r="19" spans="1:6" s="14" customFormat="1" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="27"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+    </row>
+    <row r="20" spans="1:6" s="14" customFormat="1" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="27"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+    </row>
+    <row r="21" spans="1:6" s="14" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="27"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+    </row>
+    <row r="22" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="F22" s="25" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="F23" s="18" t="s">
+    <row r="23" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="F23" s="15" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="F24" s="19" t="s">
+    <row r="24" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="F24" s="16" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:6" s="16" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F25" s="20" t="s">
+    <row r="25" spans="1:6" s="14" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F25" s="17" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:6" s="16" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="1:6" s="16" customFormat="1" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="21" t="s">
+    <row r="26" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:6" s="14" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:6" s="14" customFormat="1" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B30" s="22"/>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="23"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="20"/>
     </row>
     <row r="35" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B35" s="11"/>
-      <c r="C35" s="13"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="12"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="12"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="12"/>
+      <c r="F35" s="11"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C36" s="12"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
     </row>
     <row r="38" spans="1:6" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="B38" s="14" t="s">
+      <c r="B38" s="13" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregando plano de fondo como imagen nativa
</commit_message>
<xml_diff>
--- a/plantilla_presupuesto.xlsx
+++ b/plantilla_presupuesto.xlsx
@@ -568,72 +568,6 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>2509024</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="Rectángulo 6"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="10942134" cy="8154329"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:blipFill dpi="0" rotWithShape="1">
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-            <a:alphaModFix amt="14000"/>
-          </a:blip>
-          <a:srcRect/>
-          <a:stretch>
-            <a:fillRect/>
-          </a:stretch>
-        </a:blipFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="50000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -655,7 +589,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -670,6 +604,50 @@
         <a:xfrm>
           <a:off x="4629151" y="0"/>
           <a:ext cx="1514476" cy="1514476"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>20466</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>162622</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="10974216" cy="10407805"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Ajustando margenes y centrado para PDF mas grande
</commit_message>
<xml_diff>
--- a/plantilla_presupuesto.xlsx
+++ b/plantilla_presupuesto.xlsx
@@ -621,9 +621,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>20466</xdr:colOff>
-      <xdr:row>43</xdr:row>
-      <xdr:rowOff>162622</xdr:rowOff>
+      <xdr:colOff>23232</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>132706</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -647,7 +647,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="10974216" cy="10407805"/>
+          <a:ext cx="10976982" cy="11051608"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1031,7 +1031,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:6" s="24" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" s="24" customFormat="1" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="26"/>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
@@ -1039,7 +1039,7 @@
       <c r="E18" s="26"/>
       <c r="F18" s="26"/>
     </row>
-    <row r="19" spans="1:6" s="14" customFormat="1" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" s="14" customFormat="1" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="27"/>
       <c r="B19" s="27"/>
       <c r="C19" s="27"/>
@@ -1047,7 +1047,7 @@
       <c r="E19" s="27"/>
       <c r="F19" s="27"/>
     </row>
-    <row r="20" spans="1:6" s="14" customFormat="1" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" s="14" customFormat="1" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="27"/>
       <c r="B20" s="27"/>
       <c r="C20" s="27"/>
@@ -1055,7 +1055,7 @@
       <c r="E20" s="27"/>
       <c r="F20" s="27"/>
     </row>
-    <row r="21" spans="1:6" s="14" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" s="14" customFormat="1" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="27"/>
       <c r="B21" s="27"/>
       <c r="C21" s="27"/>

</xml_diff>

<commit_message>
Moviendo etiquetas de totales a la columna E
</commit_message>
<xml_diff>
--- a/plantilla_presupuesto.xlsx
+++ b/plantilla_presupuesto.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
   <si>
     <t>Fecha</t>
   </si>
@@ -140,6 +140,9 @@
   <si>
     <t>¡Gracias por confiar en nosotros!</t>
   </si>
+  <si>
+    <t>*******</t>
+  </si>
 </sst>
 </file>
 
@@ -176,19 +179,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="8"/>
-      <color theme="1"/>
-      <name val="Century Gothic"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="7"/>
-      <color theme="1"/>
-      <name val="Century Gothic"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -240,6 +230,19 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial Black"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Century Gothic"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -275,7 +278,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -360,43 +363,6 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
@@ -478,7 +444,9 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -490,64 +458,101 @@
   </cellStyleXfs>
   <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -570,26 +575,26 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>3048001</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>11616</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>304802</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>180976</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>34848</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>69695</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1"/>
+        <xdr:cNvPr id="3" name="Imagen 2"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -602,8 +607,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4629151" y="0"/>
-          <a:ext cx="1514476" cy="1514476"/>
+          <a:off x="11616" y="0"/>
+          <a:ext cx="9699238" cy="10976982"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -614,26 +619,26 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2079238</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>11616</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>23232</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>132706</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>699742</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>13014</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2"/>
+        <xdr:cNvPr id="2" name="Imagen 1"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -646,12 +651,18 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="10976982" cy="11051608"/>
+          <a:off x="3658994" y="11616"/>
+          <a:ext cx="2082028" cy="2045788"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom prst="ellipse">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst>
+          <a:softEdge rad="112500"/>
+        </a:effectLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -925,195 +936,204 @@
   <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="37.85546875" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52" style="2" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.5703125" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="2"/>
+      <c r="A1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="25" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="24" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="24" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="24" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="24" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="24" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="16" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="17" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="D17" s="22" t="s">
+      <c r="D17" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E17" s="22" t="s">
+      <c r="E17" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="F17" s="23" t="s">
+      <c r="F17" s="10" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:6" s="24" customFormat="1" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="26"/>
-      <c r="B18" s="26"/>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
+    <row r="18" spans="1:6" s="12" customFormat="1" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
     </row>
     <row r="19" spans="1:6" s="14" customFormat="1" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="27"/>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
+      <c r="A19" s="13"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
     </row>
     <row r="20" spans="1:6" s="14" customFormat="1" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="27"/>
-      <c r="B20" s="27"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-    </row>
-    <row r="21" spans="1:6" s="14" customFormat="1" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="27"/>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
+      <c r="A20" s="13"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+    </row>
+    <row r="21" spans="1:6" s="14" customFormat="1" ht="77.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
     </row>
     <row r="22" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="F22" s="25" t="s">
+      <c r="E22" s="23" t="s">
         <v>21</v>
       </c>
+      <c r="F22" s="23"/>
     </row>
     <row r="23" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="F23" s="15" t="s">
+      <c r="E23" s="15" t="s">
         <v>10</v>
       </c>
+      <c r="F23" s="15"/>
     </row>
     <row r="24" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="F24" s="16" t="s">
+      <c r="E24" s="16" t="s">
         <v>22</v>
       </c>
+      <c r="F24" s="16"/>
     </row>
     <row r="25" spans="1:6" s="14" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F25" s="17" t="s">
+      <c r="E25" s="17" t="s">
         <v>23</v>
       </c>
+      <c r="F25" s="17"/>
     </row>
     <row r="26" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:6" s="14" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="1:6" s="14" customFormat="1" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="18" t="s">
+    <row r="29" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:6" s="14" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="20"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
     </row>
     <row r="35" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B35" s="10"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="12"/>
-      <c r="E35" s="12"/>
-      <c r="F35" s="11"/>
+      <c r="B35" s="19"/>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
+      <c r="F35" s="21"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
     </row>
     <row r="38" spans="1:6" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="B38" s="13" t="s">
+      <c r="B38" s="22" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Version final definitiva con blindaje visual completo
</commit_message>
<xml_diff>
--- a/plantilla_presupuesto.xlsx
+++ b/plantilla_presupuesto.xlsx
@@ -581,10 +581,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>34848</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>127775</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1231280</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>127774</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -608,7 +608,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="11616" y="0"/>
-          <a:ext cx="9699238" cy="10976982"/>
+          <a:ext cx="9827012" cy="11360304"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -626,7 +626,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>699742</xdr:colOff>
+      <xdr:colOff>525504</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>13014</xdr:rowOff>
     </xdr:to>
@@ -937,7 +937,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52" style="2" customWidth="1"/>
+    <col min="2" max="2" width="54.5703125" style="2" customWidth="1"/>
     <col min="3" max="3" width="11.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.7109375" style="2" bestFit="1" customWidth="1"/>

</xml_diff>